<commit_message>
Fix Excel intake workbook compatibility
</commit_message>
<xml_diff>
--- a/intake/phner-intake.xlsx
+++ b/intake/phner-intake.xlsx
@@ -679,133 +679,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Entities" displayName="Entities" ref="A1:O2" headerRowCount="1">
-  <autoFilter ref="A1:O2"/>
-  <tableColumns count="15">
-    <tableColumn id="1" name="intake_key *"/>
-    <tableColumn id="2" name="preferred_name *"/>
-    <tableColumn id="3" name="entity_type *"/>
-    <tableColumn id="4" name="status *"/>
-    <tableColumn id="5" name="assertion_status *"/>
-    <tableColumn id="6" name="steward *"/>
-    <tableColumn id="7" name="classifications"/>
-    <tableColumn id="8" name="jurisdiction_scopes"/>
-    <tableColumn id="9" name="valid_from"/>
-    <tableColumn id="10" name="valid_to"/>
-    <tableColumn id="11" name="official_urls"/>
-    <tableColumn id="12" name="source_keys"/>
-    <tableColumn id="13" name="reviewed_by"/>
-    <tableColumn id="14" name="last_reviewed"/>
-    <tableColumn id="15" name="notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Relationships" displayName="Relationships" ref="A1:M2" headerRowCount="1">
-  <autoFilter ref="A1:M2"/>
-  <tableColumns count="13">
-    <tableColumn id="1" name="intake_key *"/>
-    <tableColumn id="2" name="subject_intake_key *"/>
-    <tableColumn id="3" name="relationship_type *"/>
-    <tableColumn id="4" name="object_intake_key *"/>
-    <tableColumn id="5" name="valid_from"/>
-    <tableColumn id="6" name="valid_to"/>
-    <tableColumn id="7" name="source_keys *"/>
-    <tableColumn id="8" name="assertion_status *"/>
-    <tableColumn id="9" name="steward *"/>
-    <tableColumn id="10" name="identity_reviewed_by"/>
-    <tableColumn id="11" name="identity_reviewed_at"/>
-    <tableColumn id="12" name="identity_rationale"/>
-    <tableColumn id="13" name="notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Sources" displayName="Sources" ref="A1:J2" headerRowCount="1">
-  <autoFilter ref="A1:J2"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="intake_key *"/>
-    <tableColumn id="2" name="source_type *"/>
-    <tableColumn id="3" name="title *"/>
-    <tableColumn id="4" name="publisher"/>
-    <tableColumn id="5" name="url"/>
-    <tableColumn id="6" name="document_identifier"/>
-    <tableColumn id="7" name="retrieved_at"/>
-    <tableColumn id="8" name="locator"/>
-    <tableColumn id="9" name="content_hash"/>
-    <tableColumn id="10" name="notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Names" displayName="Names" ref="A1:H2" headerRowCount="1">
-  <autoFilter ref="A1:H2"/>
-  <tableColumns count="8">
-    <tableColumn id="1" name="entity_intake_key *"/>
-    <tableColumn id="2" name="value *"/>
-    <tableColumn id="3" name="name_type *"/>
-    <tableColumn id="4" name="language"/>
-    <tableColumn id="5" name="is_official"/>
-    <tableColumn id="6" name="valid_from"/>
-    <tableColumn id="7" name="valid_to"/>
-    <tableColumn id="8" name="source_keys"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Locations" displayName="Locations" ref="A1:L2" headerRowCount="1">
-  <autoFilter ref="A1:L2"/>
-  <tableColumns count="12">
-    <tableColumn id="1" name="entity_intake_key *"/>
-    <tableColumn id="2" name="location_type"/>
-    <tableColumn id="3" name="address_lines"/>
-    <tableColumn id="4" name="locality"/>
-    <tableColumn id="5" name="administrative_area_text"/>
-    <tableColumn id="6" name="postal_code"/>
-    <tableColumn id="7" name="jurisdiction_intake_key"/>
-    <tableColumn id="8" name="latitude"/>
-    <tableColumn id="9" name="longitude"/>
-    <tableColumn id="10" name="valid_from"/>
-    <tableColumn id="11" name="valid_to"/>
-    <tableColumn id="12" name="source_keys"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PlatformParticipations" displayName="PlatformParticipations" ref="A1:N2" headerRowCount="1">
-  <autoFilter ref="A1:N2"/>
-  <tableColumns count="14">
-    <tableColumn id="1" name="intake_key *"/>
-    <tableColumn id="2" name="entity_intake_key *"/>
-    <tableColumn id="3" name="platform_intake_key *"/>
-    <tableColumn id="4" name="roles *"/>
-    <tableColumn id="5" name="lifecycle_status *"/>
-    <tableColumn id="6" name="environments"/>
-    <tableColumn id="7" name="data_exchange_modes"/>
-    <tableColumn id="8" name="capabilities"/>
-    <tableColumn id="9" name="valid_from"/>
-    <tableColumn id="10" name="valid_to"/>
-    <tableColumn id="11" name="source_keys *"/>
-    <tableColumn id="12" name="assertion_status *"/>
-    <tableColumn id="13" name="steward *"/>
-    <tableColumn id="14" name="notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RelationshipReference" displayName="RelationshipReference" ref="A1:E18" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RelationshipReference" displayName="RelationshipReference" ref="A1:E18" headerRowCount="1">
   <autoFilter ref="A1:E18"/>
   <tableColumns count="5">
     <tableColumn id="1" name="relationship_type"/>
@@ -8904,9 +8778,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -15957,9 +15828,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -20863,9 +20731,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -25563,9 +25428,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -32477,9 +32339,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -38741,9 +38600,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>